<commit_message>
feat: Integrate Model Governance & Reinsurer Ratings into Stress Testing & Forecasting; Add Interactive Notebooks; Clean up legacy agents; Add Chatbot UI improvements
</commit_message>
<xml_diff>
--- a/reports/risk_summary_report.xlsx
+++ b/reports/risk_summary_report.xlsx
@@ -10,7 +10,6 @@
     <sheet name="Portfolio Metrics" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Risks by Product" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="ML Feature Importance" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Model Governance" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -790,40 +789,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>count</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Pass - Compliant</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>2977</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>